<commit_message>
DB ENV variable change and CDR coder changes and
</commit_message>
<xml_diff>
--- a/Backend/utility/cdr_report/CDR_Pipelines/s4c1_cc_raw.xlsx
+++ b/Backend/utility/cdr_report/CDR_Pipelines/s4c1_cc_raw.xlsx
@@ -840,7 +840,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>PACKAGING is not part of the electrical or safety circuitry and does not affect safety operation.</t>
+          <t>PACKAGING is not part of the product's electrical or safety-related function.</t>
         </is>
       </c>
       <c r="V4" t="n">
@@ -1046,11 +1046,11 @@
       </c>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[4]</t>
         </is>
       </c>
       <c r="T6" t="n">
@@ -1058,17 +1058,17 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>WELDMENT WRAP is likely a mechanical support, not directly related to safety or hazardous circuitry.</t>
+          <t>WELDMENT WRAP may be part of the enclosure or shielding, preventing access to hazardous areas.</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W6" t="n">
         <v>8</v>
       </c>
       <c r="X6" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Sealing fasteners may be relied upon to maintain segregation or environmental protection, thus critical.</t>
+          <t>Sealing fasteners may be relied upon to maintain environmental or electrical segregation.</t>
         </is>
       </c>
       <c r="V7" t="n">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>CLAMP OPTICAL WINDOW may prevent access to hazardous areas or maintain enclosure integrity.</t>
+          <t>CLAMP OPTICAL WINDOW likely secures a barrier, preventing access to hazardous areas.</t>
         </is>
       </c>
       <c r="V8" t="n">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>GLASS is likely part of a viewing window, preventing access to hazardous areas.</t>
+          <t>GLASS is likely part of a window or barrier, preventing access to hazardous circuitry.</t>
         </is>
       </c>
       <c r="V9" t="n">
@@ -1470,33 +1470,33 @@
       </c>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[2, 3, 7]</t>
         </is>
       </c>
       <c r="T10" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>LED Ring PCA is not typically part of safety or hazardous circuitry unless used for indication in safety systems.</t>
+          <t>LED Ring PCA is a PCB, possibly in safety or hazardous circuitry, and may be relied upon for safe operation.</t>
         </is>
       </c>
       <c r="V10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W10" t="n">
         <v>8</v>
       </c>
       <c r="X10" t="n">
-        <v>0</v>
+        <v>0.375</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1575,33 +1575,33 @@
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[2, 3, 7]</t>
         </is>
       </c>
       <c r="T11" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Carrier Board is a control/processing board, not directly related to safety or hazardous circuitry.</t>
+          <t>Carrier Board is a PCB, likely in hazardous or safety-related circuitry, and may be relied upon for safe operation.</t>
         </is>
       </c>
       <c r="V11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W11" t="n">
         <v>8</v>
       </c>
       <c r="X11" t="n">
-        <v>0</v>
+        <v>0.375</v>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Power Distribution PCA is likely in hazardous and safety circuitry, relied upon for safe abnormal operation.</t>
+          <t>Power Distribution PCA is a PCB in hazardous and safety-related circuitry, relied upon for safe operation.</t>
         </is>
       </c>
       <c r="V12" t="n">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>POST CAMERA is a mechanical part, not directly related to safety or hazardous circuitry.</t>
+          <t>POST CAMERA is a mechanical part, not directly related to electrical safety or hazardous circuitry.</t>
         </is>
       </c>
       <c r="V13" t="n">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>WING LOWER is a mechanical part, not directly related to safety or hazardous circuitry.</t>
+          <t>WING LOWER is a mechanical part, not directly related to electrical safety or hazardous circuitry.</t>
         </is>
       </c>
       <c r="V14" t="n">
@@ -2023,7 +2023,7 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>ARM CAMERA is a mechanical part, not directly related to safety or hazardous circuitry.</t>
+          <t>ARM CAMERA is a mechanical part, not directly related to electrical safety or hazardous circuitry.</t>
         </is>
       </c>
       <c r="V15" t="n">
@@ -2116,33 +2116,33 @@
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[2, 3, 7]</t>
         </is>
       </c>
       <c r="T16" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>Camera is not part of safety or hazardous circuitry, unless used for safety monitoring (not indicated here).</t>
+          <t>Camera is an electronic device, likely in hazardous or safety-related circuitry, and may be relied upon for safe operation.</t>
         </is>
       </c>
       <c r="V16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W16" t="n">
         <v>8</v>
       </c>
       <c r="X16" t="n">
-        <v>0</v>
+        <v>0.375</v>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2233,11 +2233,11 @@
         </is>
       </c>
       <c r="T17" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>ARM STIFFENER is a mechanical support part, not directly related to safety or hazardous circuitry.</t>
+          <t>ARM STIFFENER is a mechanical support component, not associated with safety, hazardous, or spacing functions.</t>
         </is>
       </c>
       <c r="V17" t="n">
@@ -2342,11 +2342,11 @@
         </is>
       </c>
       <c r="T18" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>WING UPPER is a structural component, not enclosing or segregating hazardous circuitry.</t>
+          <t>WING UPPER is a structural/mechanical part, not enclosing hazardous circuitry or maintaining safety spacings.</t>
         </is>
       </c>
       <c r="V18" t="n">
@@ -2439,11 +2439,11 @@
         </is>
       </c>
       <c r="T19" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Damper, Sandwich Mount is for vibration isolation, not directly related to electrical safety or hazardous circuitry.</t>
+          <t>Damper, Sandwich Mount is for vibration isolation, not for safety, hazardous, or spacing/segregation functions.</t>
         </is>
       </c>
       <c r="V19" t="n">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2532,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>[2, 3, 7]</t>
+          <t>[3, 7]</t>
         </is>
       </c>
       <c r="T20" t="n">
@@ -2540,17 +2540,17 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Ground Strap is essential for grounding, located in safety/hazardous circuitry, and relied upon for safe abnormal operation.</t>
+          <t>Ground Strap, Braided Copper is likely part of protective earthing; failure could result in hazardous voltages on accessible parts.</t>
         </is>
       </c>
       <c r="V20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W20" t="n">
         <v>8</v>
       </c>
       <c r="X20" t="n">
-        <v>0.375</v>
+        <v>0.25</v>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
@@ -2649,7 +2649,7 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>COVER TOP likely encloses hazardous circuitry, preventing access and providing protection.</t>
+          <t>COVER TOP likely encloses hazardous circuitry, preventing user access to dangerous voltages or moving parts.</t>
         </is>
       </c>
       <c r="V21" t="n">
@@ -2742,11 +2742,11 @@
         </is>
       </c>
       <c r="T22" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Indicating Desiccant Canister is for moisture control, not directly related to electrical safety or hazardous circuitry.</t>
+          <t>Indicating Desiccant Canister is for moisture control, not related to electrical safety or hazardous circuit access.</t>
         </is>
       </c>
       <c r="V22" t="n">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2851,11 +2851,11 @@
         </is>
       </c>
       <c r="T23" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>BRACKET CAMERA SUPPORT is a mechanical support, not involved in safety or hazardous circuitry.</t>
+          <t>BRACKET CAMERA SUPPORT is a mechanical support, not involved in safety, hazardous, or spacing/segregation functions.</t>
         </is>
       </c>
       <c r="V23" t="n">
@@ -2869,7 +2869,7 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2952,11 +2952,11 @@
         </is>
       </c>
       <c r="T24" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Lens is an optical component, not related to electrical safety or hazardous circuitry.</t>
+          <t>Lens is an optical component, not related to electrical safety or hazardous circuit access.</t>
         </is>
       </c>
       <c r="V24" t="n">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3045,11 +3045,11 @@
         </is>
       </c>
       <c r="T25" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Optical Filter is not involved in electrical safety or hazardous circuitry.</t>
+          <t>Optical Filter is not related to electrical safety, hazardous circuits, or spacing/segregation.</t>
         </is>
       </c>
       <c r="V25" t="n">
@@ -3063,7 +3063,7 @@
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3154,11 +3154,11 @@
         </is>
       </c>
       <c r="T26" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>TIM CAMERA is a functional device, but not directly related to safety or hazardous circuitry.</t>
+          <t>TIM CAMERA is a functional module, not specifically identified as safety or hazardous circuit related.</t>
         </is>
       </c>
       <c r="V26" t="n">
@@ -3172,7 +3172,7 @@
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3263,11 +3263,11 @@
         </is>
       </c>
       <c r="T27" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>MOUNT TRIPOD is a mechanical support, not related to safety or hazardous circuitry.</t>
+          <t>MOUNT TRIPOD is a mechanical support, not enclosing hazardous circuitry or maintaining safety spacings.</t>
         </is>
       </c>
       <c r="V27" t="n">
@@ -3281,7 +3281,7 @@
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3356,25 +3356,25 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>[5, 7]</t>
+          <t>[5]</t>
         </is>
       </c>
       <c r="T28" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>O-ring may be used to maintain environmental sealing and segregation, relied upon for safe abnormal operation.</t>
+          <t>O-ring may be used for environmental sealing, possibly maintaining required spacings or ingress protection; classified as critical conservatively.</t>
         </is>
       </c>
       <c r="V28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W28" t="n">
         <v>8</v>
       </c>
       <c r="X28" t="n">
-        <v>0.25</v>
+        <v>0.125</v>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
@@ -3469,11 +3469,11 @@
         </is>
       </c>
       <c r="T29" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>TIM XIMEA CARRIER is a mechanical carrier, not directly related to safety or hazardous circuitry.</t>
+          <t>TIM XIMEA CARRIER is a mechanical carrier, not directly related to safety, hazardous circuits, or spacing.</t>
         </is>
       </c>
       <c r="V29" t="n">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3562,25 +3562,25 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>[5, 7]</t>
+          <t>[5]</t>
         </is>
       </c>
       <c r="T30" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Sealing screw may be used to maintain enclosure integrity and segregation, relied upon for safe abnormal operation.</t>
+          <t>PAN HEAD SCREW, SEALING type, may be used to maintain environmental sealing or required spacings; classified as critical conservatively.</t>
         </is>
       </c>
       <c r="V30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W30" t="n">
         <v>8</v>
       </c>
       <c r="X30" t="n">
-        <v>0.25</v>
+        <v>0.125</v>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
@@ -3667,33 +3667,33 @@
       </c>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[3, 5]</t>
         </is>
       </c>
       <c r="T31" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>BRACKET BRAID RETENTION is a mechanical support, not directly related to safety or hazardous circuitry.</t>
+          <t>BRACKET BRAID RETENTION likely secures ground braids, which are part of protective earthing and may maintain spacing/segregation.</t>
         </is>
       </c>
       <c r="V31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W31" t="n">
         <v>8</v>
       </c>
       <c r="X31" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3788,7 +3788,7 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>BASE KICKSTAND is a mechanical support, not involved in safety or hazardous circuitry, nor does it maintain electrical spacings or prevent access to hazardous areas.</t>
+          <t>BASE KICKSTAND is a mechanical support part, not involved in safety or hazardous circuitry, nor does it maintain spacings or prevent access to hazardous areas.</t>
         </is>
       </c>
       <c r="V32" t="n">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>CLAMP KICKSTAND is a mechanical part for support, not related to electrical safety or hazardous circuitry.</t>
+          <t>CLAMP KICKSTAND is a mechanical component for securing the kickstand, not related to electrical safety or hazardous circuitry.</t>
         </is>
       </c>
       <c r="V33" t="n">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>ROD KICKSTAND is a mechanical component, not involved in safety or hazardous electrical functions.</t>
+          <t>ROD KICKSTAND is a structural part, not involved in safety or hazardous electrical functions.</t>
         </is>
       </c>
       <c r="V34" t="n">
@@ -4418,7 +4418,7 @@
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>Gasket, EMI, 2.5x1.5mm is for EMI shielding, not directly related to electrical safety or hazardous circuitry. If EMI is critical for safety, re-evaluate.</t>
+          <t>Gasket, EMI, 2.5x1.5mm is for EMI shielding, not directly related to electrical safety or hazardous circuitry. If EMI affects safety, re-evaluate.</t>
         </is>
       </c>
       <c r="V38" t="n">
@@ -4737,11 +4737,11 @@
         </is>
       </c>
       <c r="T41" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>Cable, Assembly, 0.05" Pitch, 30pos, 4.00" Long is a signal cable, not part of safety or hazardous circuitry.</t>
+          <t>Cable, Assembly, 0.05" Pitch, 30pos, 4.00" Long is a signal cable, not part of safety or hazardous circuitry unless used in such context.</t>
         </is>
       </c>
       <c r="V41" t="n">
@@ -4842,11 +4842,11 @@
         </is>
       </c>
       <c r="T42" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>Cable, Assembly, 0.05" Pitch, 40pos, 4.00" Long is a signal cable, not part of safety or hazardous circuitry.</t>
+          <t>Cable, Assembly, 0.05" Pitch, 40pos, 4.00" Long is a signal cable, not part of safety or hazardous circuitry unless used in such context.</t>
         </is>
       </c>
       <c r="V42" t="n">
@@ -4935,15 +4935,15 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>[3, 7]</t>
+          <t>[3, 8]</t>
         </is>
       </c>
       <c r="T43" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>Cord, IEC C13 to NEMA 5-15, 9.5ft connects mains power, located in hazardous circuitry and relied upon for safe abnormal operation (e.g., insulation, plug type).</t>
+          <t>Cord, IEC C13 to NEMA 5-15, 9.5ft is part of mains power connection, located in hazardous circuitry, and changing it could introduce safety hazards.</t>
         </is>
       </c>
       <c r="V43" t="n">
@@ -5044,11 +5044,11 @@
         </is>
       </c>
       <c r="T44" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>USB HUB/Splitter is a data accessory, not involved in safety or hazardous electrical functions.</t>
+          <t>USB HUB/Splitter is a data accessory, not involved in safety or hazardous circuitry.</t>
         </is>
       </c>
       <c r="V44" t="n">
@@ -5149,7 +5149,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>[2, 3, 7]</t>
+          <t>[2, 3, 8]</t>
         </is>
       </c>
       <c r="T45" t="n">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>ASM POWER is likely a power supply assembly, located in hazardous and safety circuitry, relied upon for safe abnormal operation.</t>
+          <t>ASM POWER is likely the main power assembly, located in hazardous and safety circuitry, and is relied upon for safe operation.</t>
         </is>
       </c>
       <c r="V45" t="n">
@@ -5258,7 +5258,7 @@
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>[2, 7]</t>
+          <t>[2, 7, 8]</t>
         </is>
       </c>
       <c r="T46" t="n">
@@ -5266,17 +5266,17 @@
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>ASM POWER BUTTON is part of safety circuitry, relied upon for safe abnormal operation (e.g., emergency shutoff).</t>
+          <t>ASM POWER BUTTON is part of safety control (power on/off), relied upon for safe abnormal operation, and its removal could introduce hazards.</t>
         </is>
       </c>
       <c r="V46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W46" t="n">
         <v>8</v>
       </c>
       <c r="X46" t="n">
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Y46" t="inlineStr">
         <is>
@@ -5375,7 +5375,7 @@
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>ASM LED POWER likely interfaces with hazardous voltages and is part of the power/safety circuit. Power assemblies are typically required by standards and relied upon for safe operation.</t>
+          <t>ASM LED POWER likely supplies power to LEDs, which may be in hazardous or safety-related circuits. Power assemblies are typically required by standards and relied upon for safe operation.</t>
         </is>
       </c>
       <c r="V47" t="n">
@@ -5484,7 +5484,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>ASM FAN may be required for thermal safety and abnormal operation. If removed, overheating could occur. Conservatively classified as critical.</t>
+          <t>ASM FAN may be required for thermal management; failure could lead to unsafe overheating. Fans are often required by standards for thermal safety.</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5593,7 +5593,7 @@
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>Lens, serialized, may prevent access to hazardous light or voltage. Removing or changing could introduce hazards. Conservatively critical.</t>
+          <t>Lens, serialized, may prevent access to hazardous light or electrical sources. Changing or deleting could introduce hazards.</t>
         </is>
       </c>
       <c r="V49" t="n">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>TAG, Product1 Mod is a label/tag, not involved in safety or hazardous circuits.</t>
+          <t>TAG, Product1 Mod is likely an identification or marking tag, not involved in safety or hazardous circuits.</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -5807,11 +5807,11 @@
         </is>
       </c>
       <c r="T51" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>GASKET-BASE-COVER-EPDM likely maintains enclosure integrity and spacings, preventing access to hazardous parts.</t>
+          <t>GASKET-BASE-COVER-EPDM may provide enclosure sealing, maintaining spacing and preventing access to hazardous parts.</t>
         </is>
       </c>
       <c r="V51" t="n">
@@ -5825,7 +5825,7 @@
       </c>
       <c r="Y51" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -5920,7 +5920,7 @@
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>GASKET LENS WINDOW SIL likely maintains enclosure integrity and prevents access to hazardous areas. Conservatively critical.</t>
+          <t>GASKET LENS WINDOW SIL likely seals the lens, preventing ingress and access to hazardous areas, and maintains required spacings.</t>
         </is>
       </c>
       <c r="V52" t="n">
@@ -6009,7 +6009,7 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>[5]</t>
+          <t>[4, 5]</t>
         </is>
       </c>
       <c r="T53" t="n">
@@ -6017,17 +6017,17 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>Sealing washer may be used to maintain environmental or electrical spacings. If changed, ingress or breakdown could occur.</t>
+          <t>Sealing washer may be critical for maintaining enclosure integrity and spacing, preventing access to hazardous parts.</t>
         </is>
       </c>
       <c r="V53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W53" t="n">
         <v>8</v>
       </c>
       <c r="X53" t="n">
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Y53" t="inlineStr">
         <is>
@@ -6114,7 +6114,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>Handle is not involved in safety, hazardous circuits, or enclosure integrity.</t>
+          <t>Handle, Folding Pull is a mechanical part for handling, not involved in safety or hazardous circuits.</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>[5]</t>
+          <t>[4, 5]</t>
         </is>
       </c>
       <c r="T55" t="n">
@@ -6211,17 +6211,17 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>Sealing screws may maintain enclosure integrity and spacings. If changed, could affect ingress protection.</t>
+          <t>Sealing screws may be relied upon to maintain enclosure integrity and prevent access to hazardous areas.</t>
         </is>
       </c>
       <c r="V55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W55" t="n">
         <v>8</v>
       </c>
       <c r="X55" t="n">
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Y55" t="inlineStr">
         <is>
@@ -6320,7 +6320,7 @@
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>TIM-LED-PCA appears to be a thermal interface material for LEDs, not directly involved in safety or hazardous circuits.</t>
+          <t>TIM-LED-PCA appears to be a thermal interface material for LEDs; unless specifically required for safety, not critical.</t>
         </is>
       </c>
       <c r="V56" t="n">
@@ -6425,7 +6425,7 @@
       </c>
       <c r="U57" t="inlineStr">
         <is>
-          <t>Kapton discs are likely for insulation or assembly aid, not relied upon for safety or hazardous circuit protection.</t>
+          <t>Kapton discs are likely for insulation or marking; unless used for safety spacings, not critical.</t>
         </is>
       </c>
       <c r="V57" t="n">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="U58" t="inlineStr">
         <is>
-          <t>TIM-BRAID-ENCLOSURE is likely a thermal interface material, not directly involved in safety or hazardous circuits.</t>
+          <t>TIM-BRAID-ENCLOSURE is likely a thermal interface material; unless used for safety or hazardous circuit segregation, not critical.</t>
         </is>
       </c>
       <c r="V58" t="n">
@@ -6631,7 +6631,7 @@
       </c>
       <c r="U59" t="inlineStr">
         <is>
-          <t>Standard nut is not relied upon for safety, hazardous circuit protection, or enclosure integrity.</t>
+          <t>Standard nut, not typically relied upon for safety or hazardous circuit segregation.</t>
         </is>
       </c>
       <c r="V59" t="n">
@@ -6728,7 +6728,7 @@
       </c>
       <c r="U60" t="inlineStr">
         <is>
-          <t>Tooth lock washer is not relied upon for safety, hazardous circuit protection, or enclosure integrity.</t>
+          <t>Tooth lock washer, standard hardware, not typically relied upon for safety or hazardous circuit segregation.</t>
         </is>
       </c>
       <c r="V60" t="n">
@@ -6825,7 +6825,7 @@
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>[5]</t>
+          <t>[4, 5]</t>
         </is>
       </c>
       <c r="T61" t="n">
@@ -6833,17 +6833,17 @@
       </c>
       <c r="U61" t="inlineStr">
         <is>
-          <t>Sealing FHCS screws may maintain enclosure integrity and spacings. If changed, could affect ingress or safety.</t>
+          <t>Sealing FHCS (flat head cap screw) may be relied upon to maintain enclosure integrity and prevent access to hazardous areas.</t>
         </is>
       </c>
       <c r="V61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W61" t="n">
         <v>8</v>
       </c>
       <c r="X61" t="n">
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Y61" t="inlineStr">
         <is>
@@ -6930,7 +6930,7 @@
       </c>
       <c r="U62" t="inlineStr">
         <is>
-          <t>Adhesive bumper is typically used for mechanical protection or vibration damping, not for electrical safety or hazardous circuit access.</t>
+          <t>Adhesive bumper is a mechanical accessory, not required for safety, spacing, or hazardous circuit protection.</t>
         </is>
       </c>
       <c r="V62" t="n">
@@ -7035,11 +7035,11 @@
         </is>
       </c>
       <c r="T63" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="U63" t="inlineStr">
         <is>
-          <t>Spring clamp for thermal strap is a mechanical fastener, not directly involved in safety or hazardous circuitry.</t>
+          <t>Spring clamp for thermal strap is a mechanical/thermal part, not directly involved in safety or hazardous circuits.</t>
         </is>
       </c>
       <c r="V63" t="n">
@@ -7144,11 +7144,11 @@
         </is>
       </c>
       <c r="T64" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="U64" t="inlineStr">
         <is>
-          <t>Thermal strap clamp is a mechanical component for thermal management, not for electrical safety or hazardous circuit access.</t>
+          <t>Thermal strap clamp is a mechanical/thermal part, not used for safety, spacing, or hazardous circuit protection.</t>
         </is>
       </c>
       <c r="V64" t="n">
@@ -7245,7 +7245,7 @@
       </c>
       <c r="U65" t="inlineStr">
         <is>
-          <t>VHB tape is generally used for mounting or vibration isolation, not for electrical safety or hazardous circuit segregation.</t>
+          <t>VHB tape is typically used for mounting, not for safety, spacing, or hazardous circuit protection.</t>
         </is>
       </c>
       <c r="V65" t="n">
@@ -7346,7 +7346,7 @@
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>[5]</t>
+          <t>[2, 7]</t>
         </is>
       </c>
       <c r="T66" t="n">
@@ -7354,17 +7354,17 @@
       </c>
       <c r="U66" t="inlineStr">
         <is>
-          <t>Strain relief carrier is likely relied upon to maintain cable integrity and prevent hazardous conditions due to cable movement or stress.</t>
+          <t>Strain relief carrier is likely part of safety-related cable management, preventing hazardous stress on wiring.</t>
         </is>
       </c>
       <c r="V66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W66" t="n">
         <v>8</v>
       </c>
       <c r="X66" t="n">
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Y66" t="inlineStr">
         <is>
@@ -7451,7 +7451,7 @@
       </c>
       <c r="U67" t="inlineStr">
         <is>
-          <t>Screw (SHCS) is a general fastener, not used for safety, hazardous circuit access, or spacing/segregation in most cases.</t>
+          <t>Standard screw (SHCS) is a general fastener, not used for safety, spacing, or hazardous circuit protection.</t>
         </is>
       </c>
       <c r="V67" t="n">
@@ -7548,7 +7548,7 @@
       </c>
       <c r="U68" t="inlineStr">
         <is>
-          <t>Spacer may be used to maintain required spacings or segregation between components, which can be critical for safety compliance.</t>
+          <t>Spacer may be used to maintain required spacings or segregation, which is a safety function.</t>
         </is>
       </c>
       <c r="V68" t="n">
@@ -7645,11 +7645,11 @@
         </is>
       </c>
       <c r="T69" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="U69" t="inlineStr">
         <is>
-          <t>SSD is a data storage device, not involved in safety, hazardous circuitry, or abnormal operation safety.</t>
+          <t>SSD is a data storage device, not involved in safety, hazardous circuits, or spacing.</t>
         </is>
       </c>
       <c r="V69" t="n">
@@ -7746,7 +7746,7 @@
       </c>
       <c r="U70" t="inlineStr">
         <is>
-          <t>Screw (BHCS) is a general fastener, not used for safety, hazardous circuit access, or spacing/segregation in most cases.</t>
+          <t>Standard screw (BHCS) is a general fastener, not used for safety, spacing, or hazardous circuit protection.</t>
         </is>
       </c>
       <c r="V70" t="n">
@@ -7851,11 +7851,11 @@
         </is>
       </c>
       <c r="T71" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="U71" t="inlineStr">
         <is>
-          <t>Power supply assembly is located in hazardous and safety circuitry, and is relied upon for safe abnormal operation.</t>
+          <t>Power supply assembly is located in hazardous and safety circuitry, and is relied upon for safe operation.</t>
         </is>
       </c>
       <c r="V71" t="n">
@@ -7960,11 +7960,11 @@
         </is>
       </c>
       <c r="T72" t="n">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="U72" t="inlineStr">
         <is>
-          <t>Power extension cable is part of hazardous and safety circuitry, and is relied upon for safe abnormal operation.</t>
+          <t>Power extension cable is part of hazardous and safety circuitry, relied upon for safe operation.</t>
         </is>
       </c>
       <c r="V72" t="n">
@@ -8065,11 +8065,11 @@
         </is>
       </c>
       <c r="T73" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="U73" t="inlineStr">
         <is>
-          <t>Ferrite clamp is used for EMI suppression, not directly for safety or hazardous circuit access.</t>
+          <t>Clamp-on ferrite is for EMI suppression, not directly a safety or hazardous circuit component.</t>
         </is>
       </c>
       <c r="V73" t="n">
@@ -8166,29 +8166,29 @@
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>[4]</t>
+          <t>[4, 5, 7]</t>
         </is>
       </c>
       <c r="T74" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>Potting compound may be used to enclose or prevent access to hazardous circuitry, which is a critical safety function.</t>
+          <t>Potting compound may be used to enclose hazardous circuitry and maintain spacings, relied upon for abnormal safety.</t>
         </is>
       </c>
       <c r="V74" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W74" t="n">
         <v>8</v>
       </c>
       <c r="X74" t="n">
-        <v>0.125</v>
+        <v>0.375</v>
       </c>
       <c r="Y74" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -8267,11 +8267,11 @@
         </is>
       </c>
       <c r="T75" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>Flat washer is a general mechanical fastener, not used for safety, hazardous circuit access, or spacing/segregation in most cases.</t>
+          <t>Flat washer is a general mechanical fastener, not used for safety, spacing, or hazardous circuit protection.</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8364,11 +8364,11 @@
         </is>
       </c>
       <c r="T76" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>Hex nut is a general mechanical fastener, not used for safety, hazardous circuit access, or spacing/segregation in most cases.</t>
+          <t>Hex nut is a general mechanical fastener, not used for safety, spacing, or hazardous circuit protection.</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -8562,7 +8562,7 @@
       </c>
       <c r="U78" t="inlineStr">
         <is>
-          <t>Standard screw (PHCS, Torx) is general hardware, not specifically required for safety, spacing, or hazardous circuit enclosure based on available info.</t>
+          <t>Standard screw (PHCS, Torx) is not inherently critical unless used in a safety or hazardous enclosure, which is not specified.</t>
         </is>
       </c>
       <c r="V78" t="n">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="U79" t="inlineStr">
         <is>
-          <t>Standard screw (PHCS, Torx) is general hardware, not identified as critical for safety or hazardous circuit enclosure.</t>
+          <t>Standard screw (PHCS, Torx) is not inherently critical unless used in a safety or hazardous enclosure, which is not specified.</t>
         </is>
       </c>
       <c r="V79" t="n">
@@ -8756,7 +8756,7 @@
       </c>
       <c r="U80" t="inlineStr">
         <is>
-          <t>Standard screw (BHCS, Torx) is general hardware, not identified as critical for safety or hazardous circuit enclosure.</t>
+          <t>Standard screw (BHCS, Torx) is not inherently critical unless used in a safety or hazardous enclosure, which is not specified.</t>
         </is>
       </c>
       <c r="V80" t="n">
@@ -8853,7 +8853,7 @@
       </c>
       <c r="U81" t="inlineStr">
         <is>
-          <t>Standard screw (PHCS, Torx) is general hardware, not identified as critical for safety or hazardous circuit enclosure.</t>
+          <t>Standard screw (PHCS, Torx) is not inherently critical unless used in a safety or hazardous enclosure, which is not specified.</t>
         </is>
       </c>
       <c r="V81" t="n">
@@ -8946,11 +8946,11 @@
         </is>
       </c>
       <c r="T82" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="U82" t="inlineStr">
         <is>
-          <t>Bellville washer is typically used for preload; unless specifically used for spacing/segregation in safety circuits, it is not critical.</t>
+          <t>Bellville washer is a general hardware item, not typically relied upon for safety, spacing, or hazardous circuit enclosure unless specifically called out, which is not indicated here.</t>
         </is>
       </c>
       <c r="V82" t="n">
@@ -9055,7 +9055,7 @@
       </c>
       <c r="U83" t="inlineStr">
         <is>
-          <t>Grease is used for lubrication; unless required for hazardous circuit insulation or safety, it is not critical.</t>
+          <t>Grease is not typically critical unless used for electrical insulation or thermal interface in a safety-related application, which is not specified.</t>
         </is>
       </c>
       <c r="V83" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="U84" t="inlineStr">
         <is>
-          <t>Thermal interface material (TIM) for heat sink is not typically critical unless relied upon for abnormal operation safety or hazardous circuit insulation, which is not indicated.</t>
+          <t>Thermal Interface Material (TIM) for heat sink is not critical unless required for abnormal operation safety or hazardous circuit isolation, which is not specified.</t>
         </is>
       </c>
       <c r="V84" t="n">
@@ -9269,7 +9269,7 @@
       </c>
       <c r="U85" t="inlineStr">
         <is>
-          <t>Loctite adhesive is used for mechanical retention; not typically critical unless specifically required for safety or hazardous circuit enclosure.</t>
+          <t>Loctite adhesive is not typically critical unless used to secure safety-related or hazardous circuit components, which is not specified.</t>
         </is>
       </c>
       <c r="V85" t="n">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="U86" t="inlineStr">
         <is>
-          <t>Standard screw (PHCS, Torx) is general hardware, not identified as critical for safety or hazardous circuit enclosure.</t>
+          <t>Standard screw (PHCS, Torx) is not inherently critical unless used in a safety or hazardous enclosure, which is not specified.</t>
         </is>
       </c>
       <c r="V86" t="n">
@@ -9463,29 +9463,29 @@
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>[8]</t>
+          <t>[3, 8]</t>
         </is>
       </c>
       <c r="T87" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="U87" t="inlineStr">
         <is>
-          <t>Lithium coin battery can present a fire/explosion hazard if substituted with a non-equivalent part; conservatively classified as critical due to potential hazard.</t>
+          <t>Lithium coin battery is located in hazardous circuitry (chemical/electrical hazard) and may cause hazard if changed or deleted.</t>
         </is>
       </c>
       <c r="V87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W87" t="n">
         <v>8</v>
       </c>
       <c r="X87" t="n">
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Y87" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -9572,29 +9572,29 @@
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>[4]</t>
+          <t>[4, 8]</t>
         </is>
       </c>
       <c r="T88" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="U88" t="inlineStr">
         <is>
-          <t>Weldment may form part of the enclosure, which could prevent access to hazardous circuitry; conservatively classified as critical.</t>
+          <t>Weldment may form part of the enclosure, preventing access to hazardous circuitry; changing or deleting could create a hazard.</t>
         </is>
       </c>
       <c r="V88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W88" t="n">
         <v>8</v>
       </c>
       <c r="X88" t="n">
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Y88" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -9673,29 +9673,29 @@
       <c r="P89" t="inlineStr"/>
       <c r="Q89" t="inlineStr"/>
       <c r="R89" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[4, 8]</t>
         </is>
       </c>
       <c r="T89" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="U89" t="inlineStr">
         <is>
-          <t>Waterproof HDMI cable is not typically relied upon for safety or hazardous circuit insulation; unless used for hazardous voltage, not critical.</t>
+          <t>Waterproof bulkhead HDMI cable may be relied upon to maintain enclosure integrity and prevent access to hazardous circuits.</t>
         </is>
       </c>
       <c r="V89" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W89" t="n">
         <v>8</v>
       </c>
       <c r="X89" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="Y89" t="inlineStr">
         <is>
@@ -9778,29 +9778,29 @@
       <c r="P90" t="inlineStr"/>
       <c r="Q90" t="inlineStr"/>
       <c r="R90" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[4, 8]</t>
         </is>
       </c>
       <c r="T90" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="U90" t="inlineStr">
         <is>
-          <t>Waterproof USB3 cable is not typically relied upon for safety or hazardous circuit insulation; unless used for hazardous voltage, not critical.</t>
+          <t>Waterproof bulkhead USB3 cable may be relied upon to maintain enclosure integrity and prevent access to hazardous circuits.</t>
         </is>
       </c>
       <c r="V90" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W90" t="n">
         <v>8</v>
       </c>
       <c r="X90" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="Y90" t="inlineStr">
         <is>
@@ -9883,29 +9883,29 @@
       <c r="P91" t="inlineStr"/>
       <c r="Q91" t="inlineStr"/>
       <c r="R91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[4, 8]</t>
         </is>
       </c>
       <c r="T91" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="U91" t="inlineStr">
         <is>
-          <t>Waterproof RJ45 cable is not typically relied upon for safety or hazardous circuit insulation; unless used for hazardous voltage, not critical.</t>
+          <t>Waterproof bulkhead RJ45 cable may be relied upon to maintain enclosure integrity and prevent access to hazardous circuits.</t>
         </is>
       </c>
       <c r="V91" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W91" t="n">
         <v>8</v>
       </c>
       <c r="X91" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="Y91" t="inlineStr">
         <is>
@@ -10000,7 +10000,7 @@
       </c>
       <c r="U92" t="inlineStr">
         <is>
-          <t>Bulkhead seal cap (twist lock) is likely used to prevent access to hazardous circuitry and maintain enclosure integrity. Removing or changing it could compromise safety.</t>
+          <t>Bulkhead seal cap (twist lock) is likely used to prevent access to hazardous circuitry and maintain enclosure integrity; removal or substitution could compromise safety.</t>
         </is>
       </c>
       <c r="V92" t="n">
@@ -10101,11 +10101,11 @@
         </is>
       </c>
       <c r="T93" t="n">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="U93" t="inlineStr">
         <is>
-          <t>Waterproof bulkhead USB cable is likely used to maintain enclosure integrity and prevent access to hazardous voltages. Its removal or substitution could introduce hazards.</t>
+          <t>Waterproof bulkhead USB cable is likely part of the enclosure boundary, preventing access to hazardous voltages and maintaining ingress protection; changing or omitting could create hazards.</t>
         </is>
       </c>
       <c r="V93" t="n">
@@ -10210,7 +10210,7 @@
       </c>
       <c r="U94" t="inlineStr">
         <is>
-          <t>Bulkhead seal cap (screw lock) is used to seal and prevent access to hazardous areas. Its integrity is important for safety.</t>
+          <t>Bulkhead seal cap (screw lock) serves to prevent access to hazardous areas and maintain enclosure safety; its function is critical for user protection.</t>
         </is>
       </c>
       <c r="V94" t="n">
@@ -10307,7 +10307,7 @@
       </c>
       <c r="U95" t="inlineStr">
         <is>
-          <t>Flat washer is a general hardware item, not typically relied upon for safety or hazardous area protection unless specifically called out.</t>
+          <t>Flat washer (SS) is a general hardware item, not typically relied upon for safety or hazardous area protection unless specifically called out for spacing or segregation.</t>
         </is>
       </c>
       <c r="V95" t="n">
@@ -10416,7 +10416,7 @@
       </c>
       <c r="U96" t="inlineStr">
         <is>
-          <t>Heat sink gasket is generally for thermal management, not directly related to electrical safety or hazardous area protection.</t>
+          <t>Heat sink gasket is generally for thermal management, not directly involved in electrical safety or hazardous area protection unless special evaluation is documented.</t>
         </is>
       </c>
       <c r="V96" t="n">
@@ -10622,7 +10622,7 @@
       </c>
       <c r="U98" t="inlineStr">
         <is>
-          <t>O-ring is likely used for sealing to maintain enclosure integrity and prevent access to hazardous voltages. Its failure could compromise safety.</t>
+          <t>O-ring (large) is likely used for sealing enclosures, preventing access to hazardous voltages or ingress of contaminants; omission could compromise safety.</t>
         </is>
       </c>
       <c r="V98" t="n">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="U99" t="inlineStr">
         <is>
-          <t>O-ring is likely used for sealing to maintain enclosure integrity and prevent access to hazardous voltages. Its failure could compromise safety.</t>
+          <t>O-ring (smaller) serves a similar enclosure sealing function, maintaining protection against hazardous access or environmental ingress.</t>
         </is>
       </c>
       <c r="V99" t="n">
@@ -10816,7 +10816,7 @@
       </c>
       <c r="U100" t="inlineStr">
         <is>
-          <t>Sealing screw is likely used to maintain enclosure integrity and prevent access to hazardous areas. Its removal could compromise safety.</t>
+          <t>Sealing screw is likely used to maintain enclosure integrity and prevent access to hazardous areas; changing or omitting could create a hazard.</t>
         </is>
       </c>
       <c r="V100" t="n">
@@ -10909,11 +10909,11 @@
         </is>
       </c>
       <c r="T101" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="U101" t="inlineStr">
         <is>
-          <t>Bumper is typically for mechanical protection or vibration isolation, not directly related to electrical safety or hazardous area protection.</t>
+          <t>Bumper is typically for mechanical protection or vibration isolation, not directly involved in electrical safety or hazardous area protection.</t>
         </is>
       </c>
       <c r="V101" t="n">
@@ -11010,7 +11010,7 @@
       </c>
       <c r="U102" t="inlineStr">
         <is>
-          <t>Set screw is a general hardware item, not typically relied upon for safety or hazardous area protection unless specifically called out.</t>
+          <t>Set screw (flat tip) is a general hardware item, not typically relied upon for safety or hazardous circuit protection.</t>
         </is>
       </c>
       <c r="V102" t="n">
@@ -11107,7 +11107,7 @@
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>Sealing washer (EPDM) is likely used to maintain enclosure integrity and prevent access to hazardous voltages. Its failure could compromise safety.</t>
+          <t>Sealing washer (EPDM) is likely used to maintain enclosure sealing and prevent access to hazardous voltages; omission could compromise safety.</t>
         </is>
       </c>
       <c r="V103" t="n">
@@ -11208,11 +11208,11 @@
         </is>
       </c>
       <c r="T104" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>FPC cable is a signal cable, not typically relied upon for safety or hazardous area protection unless specifically called out.</t>
+          <t>FPC cable is a signal interconnect, not typically part of safety or hazardous circuitry unless specifically documented.</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -11317,11 +11317,11 @@
         </is>
       </c>
       <c r="T105" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>Wrap front is likely part of the enclosure, preventing access to hazardous circuitry. Its removal would compromise safety.</t>
+          <t>Wrap front is an enclosure part, directly preventing access to hazardous circuitry; removal would create a significant safety hazard.</t>
         </is>
       </c>
       <c r="V105" t="n">
@@ -11426,11 +11426,11 @@
         </is>
       </c>
       <c r="T106" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="U106" t="inlineStr">
         <is>
-          <t>Wrap back is likely part of the enclosure, preventing access to hazardous circuitry. Its removal would compromise safety.</t>
+          <t>Wrap back is an enclosure part, directly preventing access to hazardous circuitry; removal would create a significant safety hazard.</t>
         </is>
       </c>
       <c r="V106" t="n">
@@ -11539,7 +11539,7 @@
       </c>
       <c r="U107" t="inlineStr">
         <is>
-          <t>The DUCT HEATSINK likely serves as a physical barrier and may maintain spacings or prevent access to hazardous circuitry, triggering rules 4 and 5.</t>
+          <t>A duct heatsink may serve as a barrier or enclosure, preventing access to hazardous circuitry and maintaining required spacings for thermal and electrical safety.</t>
         </is>
       </c>
       <c r="V107" t="n">
@@ -11632,11 +11632,11 @@
         </is>
       </c>
       <c r="T108" t="n">
-        <v>0.95</v>
+        <v>0.6</v>
       </c>
       <c r="U108" t="inlineStr">
         <is>
-          <t>The encased magnet is not typically involved in safety or hazardous circuits, nor does it provide enclosure or spacing functions.</t>
+          <t>Encased magnet with M6 stud is unlikely to be part of safety or hazardous circuitry, nor does it typically serve a critical safety function.</t>
         </is>
       </c>
       <c r="V108" t="n">
@@ -11650,7 +11650,7 @@
       </c>
       <c r="Y108" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -11737,11 +11737,11 @@
         </is>
       </c>
       <c r="T109" t="n">
-        <v>0.98</v>
+        <v>0.7</v>
       </c>
       <c r="U109" t="inlineStr">
         <is>
-          <t>The case with foam is for packaging and not part of the operational safety or hazardous circuitry.</t>
+          <t>Case with custom foam is used for packaging and transport, not for electrical safety or hazardous circuit protection in operation.</t>
         </is>
       </c>
       <c r="V109" t="n">
@@ -11755,7 +11755,7 @@
       </c>
       <c r="Y109" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -11842,11 +11842,11 @@
         </is>
       </c>
       <c r="T110" t="n">
-        <v>0.98</v>
+        <v>0.7</v>
       </c>
       <c r="U110" t="inlineStr">
         <is>
-          <t>Poly bags are for packaging and do not impact electrical safety or hazardous circuit access.</t>
+          <t>Poly bags are for packaging and do not interact with safety or hazardous circuitry.</t>
         </is>
       </c>
       <c r="V110" t="n">
@@ -11860,7 +11860,7 @@
       </c>
       <c r="Y110" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -11947,11 +11947,11 @@
         </is>
       </c>
       <c r="T111" t="n">
-        <v>0.95</v>
+        <v>0.7</v>
       </c>
       <c r="U111" t="inlineStr">
         <is>
-          <t>Wire wrap labels are for identification and do not affect safety, hazardous circuits, or spacings.</t>
+          <t>Wire wrap labels are for identification and do not impact safety or hazardous circuit function.</t>
         </is>
       </c>
       <c r="V111" t="n">
@@ -11965,7 +11965,7 @@
       </c>
       <c r="Y111" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -12048,7 +12048,7 @@
       </c>
       <c r="S112" t="inlineStr">
         <is>
-          <t>[1, 3, 7]</t>
+          <t>[3, 7]</t>
         </is>
       </c>
       <c r="T112" t="n">
@@ -12056,17 +12056,17 @@
       </c>
       <c r="U112" t="inlineStr">
         <is>
-          <t>The AC/DC adapter is required by standards, is part of hazardous (mains) circuitry, and is relied upon for safe abnormal operation.</t>
+          <t>AC/DC adapter interfaces with mains and hazardous energy; relied upon for safe abnormal operation and is part of hazardous circuitry.</t>
         </is>
       </c>
       <c r="V112" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W112" t="n">
         <v>8</v>
       </c>
       <c r="X112" t="n">
-        <v>0.375</v>
+        <v>0.25</v>
       </c>
       <c r="Y112" t="inlineStr">
         <is>
@@ -12161,7 +12161,7 @@
       </c>
       <c r="U113" t="inlineStr">
         <is>
-          <t>The M12 sealed plug is likely used in hazardous voltage circuits and is relied upon for safe operation, especially if sealing is required.</t>
+          <t>Sealed M12 plug may be used in hazardous voltage circuits and is relied upon for safe connection integrity.</t>
         </is>
       </c>
       <c r="V113" t="n">
@@ -12258,15 +12258,15 @@
       </c>
       <c r="S114" t="inlineStr">
         <is>
-          <t>[3, 5]</t>
+          <t>[3, 7]</t>
         </is>
       </c>
       <c r="T114" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="U114" t="inlineStr">
         <is>
-          <t>Connector housing in power assembly may be used in hazardous circuits and to maintain spacings; classified as critical conservatively.</t>
+          <t>Receptacle housing for power circuits may be in hazardous voltage paths and is relied upon for safe operation.</t>
         </is>
       </c>
       <c r="V114" t="n">
@@ -12280,7 +12280,7 @@
       </c>
       <c r="Y114" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -12363,15 +12363,15 @@
       </c>
       <c r="S115" t="inlineStr">
         <is>
-          <t>[3, 5]</t>
+          <t>[3, 7]</t>
         </is>
       </c>
       <c r="T115" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="U115" t="inlineStr">
         <is>
-          <t>Crimp terminals in power assembly are likely in hazardous circuits and maintain spacings; classified as critical conservatively.</t>
+          <t>Crimp terminals for power circuits are part of hazardous voltage paths and are relied upon for safe connections.</t>
         </is>
       </c>
       <c r="V115" t="n">
@@ -12385,7 +12385,7 @@
       </c>
       <c r="Y115" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -12472,11 +12472,11 @@
         </is>
       </c>
       <c r="T116" t="n">
-        <v>0.95</v>
+        <v>0.7</v>
       </c>
       <c r="U116" t="inlineStr">
         <is>
-          <t>Wire wrap labels are for identification and do not affect safety, hazardous circuits, or spacings.</t>
+          <t>Wire wrap label is for identification and does not impact safety or hazardous circuit function.</t>
         </is>
       </c>
       <c r="V116" t="n">
@@ -12490,7 +12490,7 @@
       </c>
       <c r="Y116" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -12573,15 +12573,15 @@
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>[3, 5]</t>
+          <t>[3, 7]</t>
         </is>
       </c>
       <c r="T117" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>Circular receptacle in power assembly is likely in hazardous circuits and maintains spacings; classified as critical conservatively.</t>
+          <t>Circular receptacle for power circuits may be in hazardous voltage paths and is relied upon for safe operation.</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -12595,7 +12595,7 @@
       </c>
       <c r="Y117" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -12682,7 +12682,7 @@
         </is>
       </c>
       <c r="T118" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="U118" t="inlineStr">
         <is>
@@ -12700,7 +12700,7 @@
       </c>
       <c r="Y118" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -12787,11 +12787,11 @@
         </is>
       </c>
       <c r="T119" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="U119" t="inlineStr">
         <is>
-          <t>Crimp terminals for signal/power button are unlikely to be in hazardous or safety circuits.</t>
+          <t>Crimp terminals for power button are unlikely to be in hazardous or safety circuits.</t>
         </is>
       </c>
       <c r="V119" t="n">
@@ -12805,7 +12805,7 @@
       </c>
       <c r="Y119" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -12892,11 +12892,11 @@
         </is>
       </c>
       <c r="T120" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>Momentary button for panel is not typically in hazardous or safety circuits.</t>
+          <t>Momentary panel button is typically low voltage and not part of hazardous or safety-critical circuits.</t>
         </is>
       </c>
       <c r="V120" t="n">
@@ -12910,7 +12910,7 @@
       </c>
       <c r="Y120" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -12997,11 +12997,11 @@
         </is>
       </c>
       <c r="T121" t="n">
-        <v>0.95</v>
+        <v>0.7</v>
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>Wire wrap labels are for identification and do not affect safety, hazardous circuits, or spacings.</t>
+          <t>Wire wrap label is for identification and does not impact safety or hazardous circuit function.</t>
         </is>
       </c>
       <c r="V121" t="n">
@@ -13015,7 +13015,7 @@
       </c>
       <c r="Y121" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -13106,7 +13106,7 @@
       </c>
       <c r="U122" t="inlineStr">
         <is>
-          <t>Crimp housings are used to enclose and segregate conductors, often in hazardous or safety-related circuits. Changing or omitting could compromise spacing, insulation, or access to hazardous voltages.</t>
+          <t>Crimp housings are used to enclose and segregate conductors, often in hazardous or safety-related circuits. Failure or substitution could compromise spacing, insulation, or access prevention.</t>
         </is>
       </c>
       <c r="V122" t="n">
@@ -13211,7 +13211,7 @@
       </c>
       <c r="U123" t="inlineStr">
         <is>
-          <t>Crimp terminals are relied upon for secure electrical connections in potentially hazardous circuits. Failure or substitution could result in unsafe operation or loss of spacing/segregation.</t>
+          <t>Crimp terminals maintain electrical connections in potentially hazardous circuits and are relied upon for safe abnormal operation. Incorrect terminals can lead to overheating or arcing.</t>
         </is>
       </c>
       <c r="V123" t="n">
@@ -13316,7 +13316,7 @@
       </c>
       <c r="U124" t="inlineStr">
         <is>
-          <t>Multi-pair cable carries hazardous voltages/currents and maintains required insulation and spacing. Substitution or removal could compromise safety.</t>
+          <t>Multi-pair cable is used for power or signal transmission in hazardous circuits. It maintains spacing and insulation; substitution could affect safety margins.</t>
         </is>
       </c>
       <c r="V124" t="n">
@@ -13421,7 +13421,7 @@
       </c>
       <c r="U125" t="inlineStr">
         <is>
-          <t>Wire wrap labels are for identification and do not affect safety, spacing, or hazardous circuit access.</t>
+          <t>Wire wrap labels are for identification only and do not affect safety, spacing, or hazardous circuit access.</t>
         </is>
       </c>
       <c r="V125" t="n">
@@ -13526,7 +13526,7 @@
       </c>
       <c r="U126" t="inlineStr">
         <is>
-          <t>Wire wrap labels are for identification only and do not impact safety or hazardous circuit protection.</t>
+          <t>Wire wrap labels are for identification only and do not affect safety, spacing, or hazardous circuit access.</t>
         </is>
       </c>
       <c r="V126" t="n">
@@ -13631,7 +13631,7 @@
       </c>
       <c r="U127" t="inlineStr">
         <is>
-          <t>Crimp housing encloses and segregates conductors in hazardous circuits. Changing or omitting could compromise insulation, spacing, or access.</t>
+          <t>Crimp housings enclose and segregate conductors in hazardous circuits. They are relied upon for maintaining insulation and preventing access.</t>
         </is>
       </c>
       <c r="V127" t="n">
@@ -13728,7 +13728,7 @@
       </c>
       <c r="U128" t="inlineStr">
         <is>
-          <t>Blower with heatsink is relied upon for safe abnormal operation (thermal management). Removal or substitution could cause overheating and safety hazards.</t>
+          <t>Blower with heatsink is relied upon for safe abnormal operation (thermal management). Its failure could lead to overheating and safety hazards.</t>
         </is>
       </c>
       <c r="V128" t="n">
@@ -13825,7 +13825,7 @@
       </c>
       <c r="U129" t="inlineStr">
         <is>
-          <t>Cord grip prevents access to hazardous wiring and maintains cable strain relief and spacing. Omission could expose hazardous voltages.</t>
+          <t>Cord grip prevents access to hazardous wiring and maintains cable strain relief and spacing. Removal or substitution could compromise safety.</t>
         </is>
       </c>
       <c r="V129" t="n">
@@ -14027,7 +14027,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>Connector housing encloses hazardous conductors and maintains required spacing/segregation. Substitution could compromise safety.</t>
+          <t>Connector housing segregates and encloses hazardous conductors, maintaining insulation and preventing access.</t>
         </is>
       </c>
       <c r="V131" t="n">
@@ -14132,7 +14132,7 @@
       </c>
       <c r="U132" t="inlineStr">
         <is>
-          <t>Connector socket is relied upon for safe connection in hazardous circuits. Failure or substitution could result in unsafe operation.</t>
+          <t>Connector sockets maintain electrical connections in hazardous circuits and are relied upon for safe abnormal operation.</t>
         </is>
       </c>
       <c r="V132" t="n">
@@ -14237,7 +14237,7 @@
       </c>
       <c r="U133" t="inlineStr">
         <is>
-          <t>Wire wrap label is for identification only and does not impact safety or hazardous circuit protection.</t>
+          <t>Wire wrap labels are for identification only and do not affect safety, spacing, or hazardous circuit access.</t>
         </is>
       </c>
       <c r="V133" t="n">
@@ -14338,11 +14338,11 @@
         </is>
       </c>
       <c r="T134" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="U134" t="inlineStr">
         <is>
-          <t>Sealed plug is used in hazardous power circuits, provides insulation, spacing, and prevents access to live parts.</t>
+          <t>Sealed plug is used in power extension, likely hazardous circuit, and maintains insulation, spacing, and access prevention.</t>
         </is>
       </c>
       <c r="V134" t="n">
@@ -14447,7 +14447,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>Shielded wire carries hazardous voltages/currents and maintains required insulation and spacing. Substitution could compromise safety.</t>
+          <t>Shielded wire is used for power transmission in hazardous circuits, maintaining insulation and spacing.</t>
         </is>
       </c>
       <c r="V135" t="n">
@@ -14548,11 +14548,11 @@
         </is>
       </c>
       <c r="T136" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>Sealed plug is used in hazardous power circuits, provides insulation, spacing, and prevents access to live parts.</t>
+          <t>Sealed plug is used in power extension, likely hazardous circuit, and maintains insulation, spacing, and access prevention.</t>
         </is>
       </c>
       <c r="V136" t="n">
@@ -14653,7 +14653,7 @@
       </c>
       <c r="U137" t="inlineStr">
         <is>
-          <t>HDMI cable, even if waterproof, is not typically located in safety or hazardous circuitry, nor does it enclose hazardous areas or maintain spacings. No evidence of special evaluation or safety reliance.</t>
+          <t>HDMI cable, even if waterproof, is typically used for signal transmission and not located in safety or hazardous circuitry. It does not enclose hazardous parts or maintain spacings.</t>
         </is>
       </c>
       <c r="V137" t="n">
@@ -14754,7 +14754,7 @@
       </c>
       <c r="U138" t="inlineStr">
         <is>
-          <t>RJ45 cable, even if waterproof, is used for data/communication and not typically in safety or hazardous circuits. No indication it is relied upon for safety or spacing.</t>
+          <t>RJ45 cable, even if waterproof, is used for data communication and is not typically part of safety or hazardous circuits, nor does it provide enclosure or spacing.</t>
         </is>
       </c>
       <c r="V138" t="n">
@@ -14855,7 +14855,7 @@
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>USB extension cable is not generally used in safety or hazardous circuits, nor for spacing or enclosure. No evidence of special evaluation or safety function.</t>
+          <t>USB cable (A Male to A Female) is used for low voltage signal/power and is not generally part of safety or hazardous circuits, nor does it provide critical spacing or enclosure.</t>
         </is>
       </c>
       <c r="V139" t="n">
@@ -14944,33 +14944,33 @@
       <c r="P140" t="inlineStr"/>
       <c r="Q140" t="inlineStr"/>
       <c r="R140" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>[4, 7]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="T140" t="n">
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>Waterproof USB 3.0 cable with 22AWG power may be relied upon to prevent ingress (enclosure) and for safe abnormal operation (power handling). Conservative classification due to possible enclosure and power delivery roles.</t>
+          <t>USB 3.0 waterproof cable with 22AWG power may carry higher current, but USB 3.0 is still considered low voltage and not typically hazardous. Unless used in a safety or hazardous circuit, it is not critical.</t>
         </is>
       </c>
       <c r="V140" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W140" t="n">
         <v>8</v>
       </c>
       <c r="X140" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="Y140" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -15057,7 +15057,7 @@
       </c>
       <c r="U141" t="inlineStr">
         <is>
-          <t>USB 3.0 adapter is a passive interconnect, not typically in safety or hazardous circuits, nor used for spacing or enclosure. No evidence of safety reliance.</t>
+          <t>USB 3.0 adapter is a passive interconnect for low voltage signals and is not used for safety, hazardous circuits, or spacing/enclosure.</t>
         </is>
       </c>
       <c r="V141" t="n">
@@ -15162,7 +15162,7 @@
       </c>
       <c r="U142" t="inlineStr">
         <is>
-          <t>Desiccant canister is for moisture control, not electrical safety. Not in hazardous or safety circuits, nor used for spacing or enclosure.</t>
+          <t>Desiccant canister is for moisture control and does not interact with electrical safety, hazardous circuits, or spacing.</t>
         </is>
       </c>
       <c r="V142" t="n">
@@ -15259,7 +15259,7 @@
       </c>
       <c r="U143" t="inlineStr">
         <is>
-          <t>Duct assembly is likely for airflow, not electrical safety. No evidence it encloses hazardous circuitry or is used for spacing/segregation. If it did, more info would be needed.</t>
+          <t>ASM DUCT is likely a mechanical air duct assembly. Unless specifically used to enclose hazardous circuitry (not indicated), it is not critical.</t>
         </is>
       </c>
       <c r="V143" t="n">

</xml_diff>